<commit_message>
Rename beta -> SWITCH_RATE across model, workbook and note: 'beta' collides with equity beta in a pitch context; same parameter, same values (5.0, grid 2.5-10.3). Sensitivity CSV column and Excel labels renamed; F&F cross-references keep the beta symbol.
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9gSJbyzSDiQjZCRWxyvm1
</commit_message>
<xml_diff>
--- a/docs/nights_choice_driver.xlsx
+++ b/docs/nights_choice_driver.xlsx
@@ -773,7 +773,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Beta: share sensitivity to ln(relative price)</t>
+          <t>Switch rate: Airbnb-hotel switching per % price gap</t>
         </is>
       </c>
       <c r="B15" s="10" t="n">
@@ -2654,7 +2654,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Values computed by analysis/src/choice_nights_driver.py (same model); rows = beta, columns = Airbnb ADR growth minus hotel ADR growth per year. Static output, not formulas.</t>
+          <t>Values computed by analysis/src/choice_nights_driver.py (same model); rows = switch rate (share sensitivity to the % price gap; called beta in the F&amp;F paper), columns = Airbnb ADR growth minus hotel ADR growth per year. Static output, not formulas.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2672,7 +2672,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>beta \ ADR premium</t>
+          <t>switch rate \ ADR premium</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Merge PR #25 (guest-fee fix, take-rate path) with the validation pass; rebuild workbook
Krish's price-ratio correction is adopted as-is: PRICE_RATIO_2025 is descriptive and no
equation reads it, so no projection number moves. His note that beta_city_estimate.py's
same x1.14 defect is inconsequential is right - a constant factor shifts only the log
regression intercept, not the slope, so the null result stands unchanged.

Workbook rebuilt so the Countries and Global sheets carry his take-rate path.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9gSJbyzSDiQjZCRWxyvm1
</commit_message>
<xml_diff>
--- a/docs/nights_choice_driver.xlsx
+++ b/docs/nights_choice_driver.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration_2025" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Countries" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Calibration_2025" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Projection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Countries" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Global" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>